<commit_message>
docs(adhoc): add YAML config diff sheet to comparison
OpenShiftとKubernetesのYAML設定の違いを比較シートとして追加。
Ingress/Route、Deployment/DeploymentConfig、Namespace/Project、
securityContext/SCC、ImageStream/BuildConfigの5観点を例示。

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai_generated/adhoc/openshift_kubernetes_comparison.xlsx
+++ b/ai_generated/adhoc/openshift_kubernetes_comparison.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="OpenShift vs Kubernetes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="YAML設定の違い" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,8 +62,12 @@
       <color rgb="000563C1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -87,6 +92,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -149,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -176,6 +186,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -923,7 +939,7 @@
           <t>Kubernetes（または OKD）</t>
         </is>
       </c>
-      <c r="C30" s="8" t="n"/>
+      <c r="C30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -936,7 +952,7 @@
           <t>OpenShift</t>
         </is>
       </c>
-      <c r="C31" s="8" t="n"/>
+      <c r="C31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -949,7 +965,7 @@
           <t>OpenShift</t>
         </is>
       </c>
-      <c r="C32" s="8" t="n"/>
+      <c r="C32" s="7" t="n"/>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
@@ -1014,4 +1030,438 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>YAMLファイル内の設定の違い（Kubernetes vs OpenShift）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>OpenShift は Kubernetes 標準のマニフェスト（Deployment/Service/Namespace 等）をそのまま利用できる。違いが出るのは主に「OpenShift固有リソース」と「セキュリティ既定値」。代表的な5つを並べて示す。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>観点</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Kubernetes</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>OpenShift</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="270" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>① 外部公開
+(Ingress vs Route)
+IngressはK8s標準、
+RouteはOpenShift固有</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>apiVersion: networking.k8s.io/v1
+kind: Ingress
+metadata:
+  name: myapp
+spec:
+  ingressClassName: nginx
+  rules:
+  - host: myapp.example.com
+    http:
+      paths:
+      - path: /
+        pathType: Prefix
+        backend:
+          service:
+            name: myapp
+            port:
+              number: 8080</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>apiVersion: route.openshift.io/v1
+kind: Route
+metadata:
+  name: myapp
+spec:
+  host: myapp.example.com
+  to:
+    kind: Service
+    name: myapp
+  port:
+    targetPort: 8080
+  tls:
+    termination: edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="360" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>② デプロイ
+(Deployment vs
+DeploymentConfig)
+OpenShiftもDeployment可。
+DeploymentConfigは現在
+非推奨(deprecated)</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>apiVersion: apps/v1
+kind: Deployment
+metadata:
+  name: myapp
+spec:
+  replicas: 3
+  selector:
+    matchLabels:
+      app: myapp
+  template:
+    metadata:
+      labels:
+        app: myapp
+    spec:
+      containers:
+      - name: myapp
+        image: myapp:latest</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>apiVersion: apps.openshift.io/v1
+kind: DeploymentConfig
+metadata:
+  name: myapp
+spec:
+  replicas: 3
+  selector:
+    app: myapp        # matchLabels不要
+  template:
+    metadata:
+      labels:
+        app: myapp
+    spec:
+      containers:
+      - name: myapp
+        image: myapp:latest
+  triggers:           # OpenShift固有
+  - type: ConfigChange
+  - type: ImageChange
+    imageChangeParams:
+      automatic: true
+      containerNames: [myapp]
+      from:
+        kind: ImageStreamTag
+        name: myapp:latest</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="130" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>③ 名前空間
+(Namespace vs
+Project)
+OpenShiftはNamespaceも
+利用可。Projectは表示名・
+説明を付与できる拡張</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>apiVersion: v1
+kind: Namespace
+metadata:
+  name: myproject</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>apiVersion: project.openshift.io/v1
+kind: Project
+metadata:
+  name: myproject
+  annotations:
+    openshift.io/display-name: "My Project"</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="200" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>④ 実行ユーザー
+(securityContext)
+K8sは固定UID指定可。
+OpenShiftは既定SCCで
+UIDをレンジから自動採番
+(固定UIDは弾かれやすい)</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t># Pod側で任意の固定UIDを指定可能
+spec:
+  securityContext:
+    runAsNonRoot: true
+    runAsUser: 1000
+    fsGroup: 2000</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t># Pod側はrunAsUserを指定せず、
+# OpenShiftが割当範囲から自動採番。
+# 範囲はSCC(security.openshift.io/v1)で定義:
+runAsUser:
+  type: MustRunAsRange
+  uidRangeMin: 1000700000
+  uidRangeMax: 1000709999
+# 固定UIDが必須ならSCCで
+# RunAsAny等の許可が必要</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="300" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>⑤ ビルド/イメージ管理
+(ImageStream・
+BuildConfig)
+OpenShift固有。
+Kubernetesに同等リソース
+なし(外部CI/レジストリで代替)</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t># Kubernetesには該当リソースなし。
+# 外部CI(GitHub Actions等)で
+# イメージをビルドし、外部レジストリ
+# (Docker Hub/ECR/GCR等)へpush。
+# Deploymentのimage:で参照する。</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>apiVersion: image.openshift.io/v1
+kind: ImageStream
+metadata:
+  name: myapp
+---
+apiVersion: build.openshift.io/v1
+kind: BuildConfig
+metadata:
+  name: myapp
+spec:
+  source:
+    type: Git
+    git:
+      uri: https://github.com/org/myapp
+  strategy:
+    type: Source        # S2Iビルド
+  output:
+    to:
+      kind: ImageStreamTag
+      name: myapp:latest</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>■ apiVersion / kind の対応early表</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Kubernetes (kind / apiVersion)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>OpenShift (kind / apiVersion)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>外部公開</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Ingress / networking.k8s.io/v1</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Route / route.openshift.io/v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>デプロイ</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Deployment / apps/v1</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>DeploymentConfig / apps.openshift.io/v1（非推奨）
+※Deployment(apps/v1)も利用可</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>名前空間</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Namespace / v1</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>Project / project.openshift.io/v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>セキュリティ</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>（PodSecurity Admission 等）</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>SecurityContextConstraints / security.openshift.io/v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>イメージ管理</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>（該当なし／外部CI・レジストリ）</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>ImageStream / image.openshift.io/v1
+BuildConfig / build.openshift.io/v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>※ DeploymentConfig は OpenShift 4.14 時点で非推奨（deprecated）。新規は標準の Deployment 推奨。※ securityContext の挙動は適用される SCC により変わる。バージョンや製品更新で差異あり、必ず公式ドキュメントで最新確認を。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Routes と Ingress の違い（OpenShift公式）: https://github.com/openshift/openshift-docs/blob/main/modules/nw-understanding-networking-routes-ingress-example.adoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>DeploymentConfig（apps.openshift.io/v1, deprecated）: https://docs.openshift.com/container-platform/latest/applications/deployments/what-deployments-are.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>SecurityContextConstraints（security.openshift.io/v1）: https://docs.openshift.com/container-platform/latest/authentication/managing-security-context-constraints.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>ImageStream / BuildConfig（S2I）: https://docs.openshift.com/container-platform/latest/cicd/builds/understanding-image-builds.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>Kubernetes Ingress 公式: https://kubernetes.io/ja/docs/concepts/services-networking/ingress/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(adhoc): add architecture and config diff sheet
クラスタ構成（ノードOS/CNI/Operator管理/プロジェクト初期構成等）と
マニフェスト設定（SCC×SA紐付け/Route詳細/Template/CLI等）の
比較シートを追加。

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai_generated/adhoc/openshift_kubernetes_comparison.xlsx
+++ b/ai_generated/adhoc/openshift_kubernetes_comparison.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="OpenShift vs Kubernetes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="YAML設定の違い" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="構成・設定の違い" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1464,4 +1465,408 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>構成・設定の違い（Kubernetes vs OpenShift）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>「クラスタアーキテクチャ構成」と「マニフェスト・運用設定」の観点で、実務でつまずきやすい差分を整理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>■ 構成（アーキテクチャ）系</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>観点</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Kubernetes</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>OpenShift</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>ノードOS</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>ノードのLinuxディストリビューションは自由（Ubuntu/RHEL/Amazon Linux等）。OS管理は利用者責任。</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>コントロールプレーン/ワーカーとも RHCOS（Red Hat CoreOS）が必須。イミュータブルOSで、OS更新もクラスタ更新に統合。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>クラスタ管理
+アーキテクチャ</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>各種アドオン（DNS, Ingress, 監視等）を個別に導入・管理。構成は利用者が組み立てる。</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Operatorベースで宣言的に管理。Cluster Version Operator が全コンポーネントのバージョン・構成を統括。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>ネットワーク
+（CNIプラグイン）</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>CNIは選択制。Calico / Cilium / Flannel 等を自分で導入・構成する。</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>OVN-Kubernetes が既定。Cluster Network Operator(operator.openshift.io/v1 Network)で構成管理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="64" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Ingress/
+ルーター構成</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Ingressコントローラ（nginx/Traefik等）を別途デプロイして公開経路を用意。</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>HAProxyベースの Router がクラスタに常駐し、Routeを処理。Ingress Operatorが管理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="56" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>レジストリ・
+認証構成</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>イメージレジストリ・認証(IdP)とも外部前提で別途構成。</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>内蔵イメージレジストリ＋OAuthサーバーが構成要素として標準同梱。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>プロジェクト
+初期構成</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Namespace作成時は空。RBAC・NetworkPolicy・クォータは自分で付与。</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Project作成時に、既定のRBACロール・SCCバインド・クォータ等が自動付与される（テンプレートで制御可）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>■ 設定（マニフェスト・運用）系</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>観点</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Kubernetes</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>OpenShift</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="72" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>デフォルトの
+リソース制御</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>ResourceQuota / LimitRange は既定では無し。必要なら自分で定義。</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>プロジェクトに ResourceQuota / LimitRange が既定設定されることが多く、未指定だとPod作成が制限される場合あり。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="64" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>NetworkPolicy
+のデフォルト</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>既定では全Pod間通信が許可。分離したい場合のみ NetworkPolicy を定義。</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>プロジェクト間分離を意識した既定ポリシーが入りやすい（マルチテナント前提の設計）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="56" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>RBAC初期
+ロール設定</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>ClusterRole/Role を自分で設計・付与するのが基本。</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>admin / edit / view の既定ロール＋SCCバインドが標準。`oc adm policy` で管理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="200" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>SCCと
+ServiceAccount
+の紐付け
+(OpenShift固有)</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t># Kubernetesに同等概念なし。
+# Pod Security Admission(namespaceラベル)で
+# privileged/baseline/restricted を制御:
+apiVersion: v1
+kind: Namespace
+metadata:
+  name: myproject
+  labels:
+    pod-security.kubernetes.io/enforce: restricted</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t># どのSCCをどのServiceAccountに許可するか設定。
+# 例: anyuid SCC を SA に付与
+oc adm policy add-scc-to-user \
+  anyuid -z myapp-sa -n myproject
+# SCC本体(security.openshift.io/v1)で
+# runAsUser戦略等を定義</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="210" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Routeの
+詳細設定
+(TLS終端3種)</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t># Ingressのannotation/specで設定。
+# TLSはspec.tls[].secretName 等。
+# (実装はIngressコントローラ依存)</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>apiVersion: route.openshift.io/v1
+kind: Route
+metadata:
+  name: myapp
+  annotations:
+    # タイムアウト等を細かく設定可
+    haproxy.router.openshift.io/timeout: 30s
+spec:
+  to: {kind: Service, name: myapp}
+  tls:
+    # edge / passthrough / reencrypt の3種
+    termination: edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="64" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>構成管理
+ツール</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Helm / Kustomize が主流（どちらもOpenShiftでも利用可）。</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>上記に加え、OpenShift固有の Template（template.openshift.io/v1）でパラメータ化された一式を配布可能。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="56" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>CLI操作の違い</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>kubectl。namespaceは -n フラグ、接続先は context で切替。</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>oc（kubectl上位互換）。`oc project &lt;name&gt;` でプロジェクト切替、`oc login` で認証。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>※ 既定値（クォータ/NetworkPolicy/SCC等）はクラスタの構成やバージョンに依存する。正式な設計時は、対象クラスタの実設定と公式ドキュメントの最新版を必ず確認すること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>RHCOS（ノードOS）: https://docs.openshift.com/container-platform/latest/architecture/architecture-rhcos.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>OVN-Kubernetes（既定CNI）: https://docs.openshift.com/container-platform/latest/networking/ovn_kubernetes_network_provider/about-ovn-kubernetes.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Route と TLS終端（edge/passthrough/reencrypt）: https://docs.openshift.com/container-platform/latest/networking/routes/secured-routes.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>SecurityContextConstraints の管理: https://docs.openshift.com/container-platform/latest/authentication/managing-security-context-constraints.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>OpenShift Template: https://docs.openshift.com/container-platform/latest/openshift_images/using-templates.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Kubernetes Pod Security Admission: https://kubernetes.io/docs/concepts/security/pod-security-admission/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(adhoc): add oc command reference sheet
oc help出力をカテゴリ別に整理したocコマンド一覧シートを追加。
各コマンドのkubectl対応/OpenShift固有の区別を備考列に記載。

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai_generated/adhoc/openshift_kubernetes_comparison.xlsx
+++ b/ai_generated/adhoc/openshift_kubernetes_comparison.xlsx
@@ -10,6 +10,7 @@
     <sheet name="OpenShift vs Kubernetes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="YAML設定の違い" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="構成・設定の違い" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ocコマンド一覧" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +66,22 @@
     </font>
     <font>
       <name val="Consolas"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <b val="1"/>
+      <color rgb="00C0504D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <color rgb="00404040"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -160,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -193,6 +210,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1855,8 +1881,8 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A23:C23"/>
@@ -1869,4 +1895,1310 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C92"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>oc コマンド一覧（oc help 出力ベース）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>oc は kubectl の上位互換 CLI。kubectl のサブコマンドはほぼ同名で利用でき、加えて OpenShift 固有の操作（login / project / build / route / template / adm 等）が使える。「備考」列に kubectl 対応・OpenShift固有を記載。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>■ Basic Commands（基本コマンド）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>コマンド</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>機能（説明）</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>備考（kubectl対応 / OpenShift固有）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>login</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>OpenShiftサーバーへログインする</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有（kubectlにloginなし）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>new-project</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>新しいプロジェクト（Project）の作成を要求する</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有（kubectlはcreate namespace）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>new-app</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>ソース/イメージ/テンプレートから新規アプリを作成する</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>現在のプロジェクトの概況を表示する</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有（routeやbuildを俯瞰）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>別のプロジェクトに切り替える</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有（kubectlはctx/-n）</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>projects</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>既存のプロジェクト一覧を表示する</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>explain</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>リソースのドキュメントを取得する</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>kubectl explain 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>■ Build and Deploy Commands（ビルド＆デプロイ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>コマンド</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>機能（説明）</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>備考（kubectl対応 / OpenShift固有）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>rollout</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>リソースのロールアウトを管理する</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>kubectl rollout 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>rollback</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>アプリの一部を以前のデプロイへ戻す</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有（kubectlはrollout undo）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>new-build</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>新しいビルド構成（BuildConfig）を作成する</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>start-build</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>新しいビルドを開始する</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>cancel-build</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>実行中/保留中/新規のビルドをキャンセルする</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>import-image</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>コンテナレジストリからイメージをインポートする</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有（ImageStream）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>tag</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>既存イメージをimage streamにタグ付けする</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有（ImageStream）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>■ Application Management Commands（アプリ管理）</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>コマンド</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>機能（説明）</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>備考（kubectl対応 / OpenShift固有）</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>create</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>ファイルやstdinからリソースを作成する</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>kubectl create 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>ファイル名やstdinから構成をリソースに適用する</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>kubectl apply 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>get</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>1つまたは複数のリソースを表示する</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>kubectl get 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>describe</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>特定リソースの詳細を表示する</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>kubectl describe 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>edit</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>サーバー上のリソースを編集する</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>kubectl edit 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>オブジェクトの特定機能を設定するコマンド群</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>kubectl set 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>リソースのラベルを更新する</t>
+        </is>
+      </c>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>kubectl label 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>annotate</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>リソースのアノテーションを更新する</t>
+        </is>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>kubectl annotate 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>expose</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>複製アプリをService/Routeとして公開する</t>
+        </is>
+      </c>
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>kubectl exposeあり。ocはRoute公開も可</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>delete</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>ファイル名/stdin/リソース名/ラベルでリソースを削除する</t>
+        </is>
+      </c>
+      <c r="C35" s="16" t="inlineStr">
+        <is>
+          <t>kubectl delete 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>scale</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Deployment/ReplicaSet/RC のサイズを変更する</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>kubectl scale 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>autoscale</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Deployment/DC/RS/StatefulSet/RC をオートスケールする</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>kubectl autoscaleあり。DC対応はoc独自</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>secrets</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>シークレットを管理する</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="inlineStr">
+        <is>
+          <t>★ocのサブコマンド群（kubectlはcreate secret等）</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>■ Troubleshooting and Debugging Commands（トラブルシュート＆デバッグ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>コマンド</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>機能（説明）</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>備考（kubectl対応 / OpenShift固有）</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>logs</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Pod内コンテナのログを表示する</t>
+        </is>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>kubectl logs 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>rsh</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>コンテナ内でシェルセッションを開始する</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有（簡易なリモートシェル）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>rsync</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>ローカルとPod間でファイルをコピーする</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有（rsyncベース）</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>port-forward</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>ローカルポートをPodへフォワードする</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>kubectl port-forward 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>debug</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>デバッグ用にPodの新規インスタンスを起動する</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>kubectl debugあり</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>exec</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>コンテナ内でコマンドを実行する</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>kubectl exec 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="14" t="inlineStr">
+        <is>
+          <t>proxy</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Kubernetes APIサーバーへのプロキシを起動する</t>
+        </is>
+      </c>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>kubectl proxy 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>attach</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>実行中コンテナにアタッチする</t>
+        </is>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>kubectl attach 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>クラスタ上で特定イメージを実行する</t>
+        </is>
+      </c>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>kubectl run 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>cp</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>コンテナとの間でファイル/ディレクトリをコピーする</t>
+        </is>
+      </c>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>kubectl cp 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>wait</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>（実験的）リソースの特定条件を待機する</t>
+        </is>
+      </c>
+      <c r="C52" s="16" t="inlineStr">
+        <is>
+          <t>kubectl wait 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>イベントを一覧表示する</t>
+        </is>
+      </c>
+      <c r="C53" s="16" t="inlineStr">
+        <is>
+          <t>kubectl events 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>■ Advanced Commands（高度なコマンド）</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>コマンド</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>機能（説明）</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>備考（kubectl対応 / OpenShift固有）</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="14" t="inlineStr">
+        <is>
+          <t>adm</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>クラスタ管理ツール（管理者向けサブコマンド）</t>
+        </is>
+      </c>
+      <c r="C57" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有（oc adm policy等）</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
+        <is>
+          <t>replace</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>ファイル名/stdinでリソースを置換する</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>kubectl replace 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="14" t="inlineStr">
+        <is>
+          <t>patch</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>リソースのフィールドを更新する</t>
+        </is>
+      </c>
+      <c r="C59" s="16" t="inlineStr">
+        <is>
+          <t>kubectl patch 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>テンプレートをリソースのリストへ展開する</t>
+        </is>
+      </c>
+      <c r="C60" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有（Template）</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t>extract</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>シークレット/ConfigMapをディスクに抽出する</t>
+        </is>
+      </c>
+      <c r="C61" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>observe</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>（実験的）リソース変更を監視し反応する</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>認可ポリシーを管理する</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有（SCC/RBAC操作）</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t>auth</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>認可を検査する</t>
+        </is>
+      </c>
+      <c r="C64" s="16" t="inlineStr">
+        <is>
+          <t>kubectl auth 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="14" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>イメージ管理に役立つコマンド群</t>
+        </is>
+      </c>
+      <c r="C65" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="14" t="inlineStr">
+        <is>
+          <t>registry</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>内蔵レジストリ操作コマンド群</t>
+        </is>
+      </c>
+      <c r="C66" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="inlineStr">
+        <is>
+          <t>idle</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>スケーラブルなリソースをアイドル化する</t>
+        </is>
+      </c>
+      <c r="C67" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>api-versions</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>サーバーが対応するAPIバージョンを group/version 形式で表示</t>
+        </is>
+      </c>
+      <c r="C68" s="16" t="inlineStr">
+        <is>
+          <t>kubectl api-versions 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>api-resources</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>サーバーが対応するAPIリソースを表示する</t>
+        </is>
+      </c>
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>kubectl api-resources 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>cluster-info</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>クラスタ情報を表示する</t>
+        </is>
+      </c>
+      <c r="C70" s="16" t="inlineStr">
+        <is>
+          <t>kubectl cluster-info 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr">
+        <is>
+          <t>diff</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>稼働中バージョンと適用予定の差分を表示する</t>
+        </is>
+      </c>
+      <c r="C71" s="16" t="inlineStr">
+        <is>
+          <t>kubectl diff 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="14" t="inlineStr">
+        <is>
+          <t>kustomize</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>ディレクトリ/URLからkustomizationをビルドする</t>
+        </is>
+      </c>
+      <c r="C72" s="16" t="inlineStr">
+        <is>
+          <t>kubectl kustomize 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>■ Settings Commands（設定コマンド）</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>コマンド</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>機能（説明）</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>備考（kubectl対応 / OpenShift固有）</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="14" t="inlineStr">
+        <is>
+          <t>get-token</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>（実験的）外部OIDC発行者からトークンを取得する</t>
+        </is>
+      </c>
+      <c r="C76" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有（exec credential plugin）</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="14" t="inlineStr">
+        <is>
+          <t>logout</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>現在のサーバーセッションを終了する</t>
+        </is>
+      </c>
+      <c r="C77" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>kubeconfigを変更する</t>
+        </is>
+      </c>
+      <c r="C78" s="16" t="inlineStr">
+        <is>
+          <t>kubectl config 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="14" t="inlineStr">
+        <is>
+          <t>whoami</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>現在のセッション情報を返す</t>
+        </is>
+      </c>
+      <c r="C79" s="15" t="inlineStr">
+        <is>
+          <t>★OpenShift固有</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>completion</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>指定シェル(bash/zsh/fish/powershell)の補完コードを出力する</t>
+        </is>
+      </c>
+      <c r="C80" s="16" t="inlineStr">
+        <is>
+          <t>kubectl completion 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>■ Other Commands（その他）</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>コマンド</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>機能（説明）</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>備考（kubectl対応 / OpenShift固有）</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="14" t="inlineStr">
+        <is>
+          <t>plugin</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>プラグインと連携するユーティリティを提供する</t>
+        </is>
+      </c>
+      <c r="C84" s="16" t="inlineStr">
+        <is>
+          <t>kubectl plugin 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="14" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>クライアントとサーバーのバージョン情報を表示する</t>
+        </is>
+      </c>
+      <c r="C85" s="16" t="inlineStr">
+        <is>
+          <t>kubectl version 相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="30" customHeight="1">
+      <c r="A87" s="9" t="inlineStr">
+        <is>
+          <t>★ = OpenShift固有（または oc 独自拡張）コマンド。それ以外は kubectl にほぼ同名・同等のコマンドが存在し、oc はその上位互換として動作する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>※ 本シートは提示された `oc help` の出力に基づく。各コマンドの詳細は `oc &lt;command&gt; --help` で確認できる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="11" t="inlineStr">
+        <is>
+          <t>OpenShift CLI（oc）リファレンス: https://docs.openshift.com/container-platform/latest/cli_reference/openshift_cli/developer-cli-commands.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="11" t="inlineStr">
+        <is>
+          <t>oc と kubectl の使い分け: https://docs.openshift.com/container-platform/latest/cli_reference/openshift_cli/getting-started-cli.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="11" t="inlineStr">
+        <is>
+          <t>kubectl コマンドリファレンス: https://kubernetes.io/docs/reference/kubectl/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A82:C82"/>
+    <mergeCell ref="A90:C90"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A74:C74"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A88:C88"/>
+    <mergeCell ref="A92:C92"/>
+    <mergeCell ref="A91:C91"/>
+    <mergeCell ref="A55:C55"/>
+    <mergeCell ref="A87:C87"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(adhoc): add major oc command options sheet
主要ocコマンド(login/new-app/new-build/process/get/rollout/
expose/adm policy等)の主要オプションを抜粋シートとして追加。
公式CLIリファレンス・利用例に基づき、完全な一覧はoc --help参照と明記。

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai_generated/adhoc/openshift_kubernetes_comparison.xlsx
+++ b/ai_generated/adhoc/openshift_kubernetes_comparison.xlsx
@@ -11,6 +11,7 @@
     <sheet name="YAML設定の違い" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="構成・設定の違い" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="ocコマンド一覧" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="主要コマンドのオプション" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3201,4 +3202,437 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>主要 oc コマンドのオプション（抜粋）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>⚠️ 本シートは「よく使う主要オプションの抜粋」です。オプションは oc のバージョンで増減するため、完全・正確な一覧は各クラスタで `oc &lt;command&gt; --help` を実行して確認してください。下表のオプションは OpenShift 公式 CLI リファレンスおよび利用例に基づきます。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>コマンド</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>主要オプション（抜粋）</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>使用例</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="130" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>login</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>-u, --username : ユーザー名
+-p, --password : パスワード
+--token        : APIトークンでログイン
+--server       : APIサーバーURL（位置引数でも可）
+--insecure-skip-tls-verify : 証明書検証を省略</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>oc login --token=&lt;token&gt; \
+  --server=https://api.example:6443
+oc login -u admin -p pass \
+  https://openshift.example:6443</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>new-project</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>--display-name : 表示名
+--description  : 説明</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>oc new-project myproject \
+  --display-name="My Project"</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="160" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>new-app</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>--name          : 生成オブジェクト名
+-l, --label     : ラベル付与
+-e, --env       : 環境変数
+--strategy      : ビルド戦略(source/docker等)
+--image-stream / --docker-image : 元イメージ
+--context-dir   : ソースのサブディレクトリ
+--search / --list : イメージ・テンプレ検索</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>oc new-app \
+  https://github.com/org/app \
+  --name=myapp -l app=myapp
+oc new-app --search php</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="110" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>new-build</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>--binary    : バイナリ入力でビルド
+--strategy  : ビルド戦略(docker/source)
+--name      : BuildConfig名
+--to        : 出力ImageStreamTag</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>oc new-build --binary \
+  --strategy=docker \
+  --name custom-builder-image</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="110" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>start-build</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>--from-dir  : ディレクトリを入力に
+--from-file : ファイルを入力に
+-F, --follow: ビルドログを追従
+--wait      : 完了まで待機</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>oc start-build myapp \
+  --from-dir=. --follow</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="110" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>-f, --filename  : テンプレートファイル
+-p, --param     : パラメータ指定(KEY=VALUE)
+--param-file    : パラメータファイル
+-o              : 出力形式</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>oc process -f tmpl.yaml \
+  -p NAME=app | oc apply -f -
+oc process -f t --param-file=env</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="130" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>get</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>-o, --output       : 出力形式(yaml/json/wide)
+-w, --watch        : 変更を監視
+-l, --selector     : ラベルセレクタ
+-A, --all-namespaces : 全namespace
+--show-labels      : ラベル表示</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>oc get pods -o wide
+oc get pods --all-namespaces
+oc get pods -l app=myapp -w</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="110" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>create / apply</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>-f, --filename  : 定義ファイル/ディレクトリ/URL
+-k, --kustomize : kustomizationから
+-o, --output    : 出力形式
+--dry-run       : 実行せず検証(client/server)</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>oc apply -f manifest.yaml
+oc create -f ./dir/
+oc apply -k ./overlay/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="120" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>rollout</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>(サブコマンド) status / history /
+  undo / restart / pause / resume
+undo --to-revision : 戻す版を指定
+status -w          : 完了まで監視</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>oc rollout status deploy/myapp
+oc rollout undo deploy/myapp \
+  --to-revision=2
+oc rollout restart deploy/myapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>scale</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>--replicas         : 希望レプリカ数
+--current-replicas : 現在数の条件(一致時のみ)
+-f, --filename     : 対象をファイルで指定</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>oc scale deploy/myapp \
+  --replicas=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="110" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>expose</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>--name      : 生成するRoute/Service名
+--hostname  : Routeのホスト名
+--port      : 対象ポート
+--selector  : 対象セレクタ</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>oc expose service myapp
+oc expose svc app \
+  --hostname app.apps.example.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="110" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>logs</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>-f, --follow    : ログを追従
+-c, --container : 対象コンテナ
+--tail          : 末尾N行
+-p, --previous  : 直前の終了コンテナ</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>oc logs -f pod/myapp -c web
+oc logs deploy/myapp --tail=100</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>rsh / exec</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>rsh -c     : 対象コンテナ
+rsh -T     : TTY割当を無効化
+exec -i, --stdin : 標準入力を渡す
+exec -t, --tty   : TTYを割当
+exec -c          : 対象コンテナ</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>oc rsh pod/myapp
+oc exec -it pod/myapp -- bash</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>debug</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>--as-user / --as-root : 実行ユーザー変更
+-t, --tty             : TTY割当
+-c                    : 対象コンテナ</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>oc debug deploy/myapp
+oc debug node/&lt;node-name&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="140" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>adm policy</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>(サブコマンド)
+  add-scc-to-user &lt;scc&gt; -z &lt;sa&gt;
+  add-role-to-user &lt;role&gt; &lt;user&gt;
+  add-cluster-role-to-user &lt;role&gt; &lt;user&gt;
+-z          : ServiceAccount指定
+-n          : namespace指定</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>oc adm policy \
+  add-scc-to-user anyuid \
+  -z myapp-sa -n myproject</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>※ グローバルオプション（全コマンド共通）: -n/--namespace, --context, --kubeconfig, --as（権限借用）, -o/--output 等。詳細は `oc options` を参照。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>OpenShift Developer CLI コマンド: https://docs.openshift.com/container-platform/latest/cli_reference/openshift_cli/developer-cli-commands.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>OpenShift Administrator CLI（oc adm）: https://docs.openshift.com/container-platform/latest/cli_reference/openshift_cli/administrator-cli-commands.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>oc new-app の使い方（公式）: https://github.com/openshift/openshift-docs/blob/main/modules/applications-create-using-cli-modify.adoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>oc process（テンプレート展開）: https://github.com/openshift/openshift-docs/blob/main/modules/templates-cli-generating-list-of-objects.adoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>kubectl コマンドリファレンス（共通オプション）: https://kubernetes.io/docs/reference/kubectl/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(adhoc): add detailed command options from real oc help
実機oc --help出力に基づくlogin/new-app/get/create/rolloutの
全オプション詳細シートを追加。バージョン正確な転記。

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai_generated/adhoc/openshift_kubernetes_comparison.xlsx
+++ b/ai_generated/adhoc/openshift_kubernetes_comparison.xlsx
@@ -12,6 +12,7 @@
     <sheet name="構成・設定の違い" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="ocコマンド一覧" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="主要コマンドのオプション" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="コマンド詳細(実出力)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -83,6 +84,29 @@
     <font>
       <name val="Yu Gothic"/>
       <color rgb="00404040"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -178,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -220,6 +244,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3635,4 +3674,1296 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B118"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>oc コマンド オプション詳細（実機 oc --help 出力ベース）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>提供された実機の `oc &lt;command&gt; --help` 出力を忠実に転記。バージョン正確（実行環境の oc に準拠）。対象コマンド: login / new-app / get / create / rollout。（他コマンドの完全な詳細が必要な場合は、同様に oc &lt;command&gt; --help の出力を提供してください）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>oc login [URL] [flags]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>サーバーへログインし、接続情報を ~/.kube/config に保存する。ユーザー名/パスワード・トークン・Webブラウザでの認証に対応。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>オプション</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>-u, --username</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>サーバーのユーザー名</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>-p, --password</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>サーバーのパスワード</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>--token</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>API サーバー認証用の Bearer トークン</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>-w, --web</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Webブラウザでログイン（OAuth2 Authorization Code Grant）。マルチユーザー環境では注意（ポートが全ユーザーに開く）</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>-c, --callback-port</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>--web 使用時のコールバックサーバーのポート（既定: ランダムな空きポート）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>--auto-open-browser</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>（実験的）ログイン時にブラウザを自動起動。--web では既定true、--exec-plugin では既定false</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>--certificate-authority</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>認証局(CA)証明書ファイルのパス</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>--insecure-skip-tls-verify</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>サーバー証明書の検証を省略（HTTPS接続が安全でなくなる）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>--exec-plugin</t>
+        </is>
+      </c>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>（実験的）外部OIDC認証に使う credentials exec plugin 種別。現状 'oc-oidc' のみ対応</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>--client-id</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>（実験的）外部OIDC issuer の Client ID（Auth Code + PKCE のみ。必須）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>--client-secret</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>（実験的）外部OIDC issuer の Client secret（任意）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>--issuer-url</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>（実験的）外部 issuer の URL（必須）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>--extra-scopes</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>（実験的）外部OIDC issuer 用の追加スコープ（任意）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>--oidc-certificate-authority</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>（実験的）外部OIDC issuer 通信時に使う CA バンドルのパス</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>oc new-app (IMAGE | IMAGESTREAM | TEMPLATE | PATH | URL ...) [flags]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>ソースコード/テンプレート/イメージから新規アプリを作成。ソースURL指定時はビルドを自動トリガー。`oc status` で進捗確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>オプション</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>--name</t>
+        </is>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>生成されるアプリのオブジェクト名</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>-l, --labels</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>このアプリの全リソースに設定するラベル</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t>-e, --env</t>
+        </is>
+      </c>
+      <c r="B27" s="21" t="inlineStr">
+        <is>
+          <t>各コンテナに設定する環境変数（KEY=VALUE）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>--env-file</t>
+        </is>
+      </c>
+      <c r="B28" s="21" t="inlineStr">
+        <is>
+          <t>各コンテナに設定する環境変数のKEY=VALUEを記載したファイル</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t>--build-env</t>
+        </is>
+      </c>
+      <c r="B29" s="21" t="inlineStr">
+        <is>
+          <t>各ビルドイメージに設定する環境変数（KEY=VALUE）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>--build-env-file</t>
+        </is>
+      </c>
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>各ビルドイメージに設定する環境変数ファイル</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>--image</t>
+        </is>
+      </c>
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>アプリに含めるコンテナイメージ名（レジストリ/リポジトリ未指定時はクライアント既定）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>-i, --image-stream</t>
+        </is>
+      </c>
+      <c r="B32" s="21" t="inlineStr">
+        <is>
+          <t>デプロイに使う既存 ImageStream 名</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>--code</t>
+        </is>
+      </c>
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>アプリのビルドに使うソースコード</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t>--context-dir</t>
+        </is>
+      </c>
+      <c r="B34" s="21" t="inlineStr">
+        <is>
+          <t>ビルドに使うソースのサブディレクトリ</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="20" t="inlineStr">
+        <is>
+          <t>--source-secret</t>
+        </is>
+      </c>
+      <c r="B35" s="21" t="inlineStr">
+        <is>
+          <t>プライベートGitリポジトリのクローンに使う既存Secret名</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="20" t="inlineStr">
+        <is>
+          <t>-f, --file</t>
+        </is>
+      </c>
+      <c r="B36" s="21" t="inlineStr">
+        <is>
+          <t>アプリに使うテンプレートファイルのパス</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="20" t="inlineStr">
+        <is>
+          <t>--template</t>
+        </is>
+      </c>
+      <c r="B37" s="21" t="inlineStr">
+        <is>
+          <t>使用する保存済みテンプレート名</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t>-p, --param</t>
+        </is>
+      </c>
+      <c r="B38" s="21" t="inlineStr">
+        <is>
+          <t>テンプレートのパラメータ値を設定/上書き（-p FOO=BAR）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="20" t="inlineStr">
+        <is>
+          <t>--param-file</t>
+        </is>
+      </c>
+      <c r="B39" s="21" t="inlineStr">
+        <is>
+          <t>テンプレートのパラメータ値を記載したファイル</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
+          <t>--strategy</t>
+        </is>
+      </c>
+      <c r="B40" s="21" t="inlineStr">
+        <is>
+          <t>ビルド戦略を明示（docker|pipeline|source）。※ pipeline は非推奨</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t>--binary</t>
+        </is>
+      </c>
+      <c r="B41" s="21" t="inlineStr">
+        <is>
+          <t>ソースURLでなくバイナリ入力を期待。トリガーは無効化される</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>--group</t>
+        </is>
+      </c>
+      <c r="B42" s="21" t="inlineStr">
+        <is>
+          <t>&lt;comp1&gt;+&lt;comp2&gt; のようにまとめるコンポーネントを指定</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>--import-mode</t>
+        </is>
+      </c>
+      <c r="B43" s="21" t="inlineStr">
+        <is>
+          <t>'PreserveOriginal' でタグの完全なmanifest listをインポート（既定 'Legacy'）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="20" t="inlineStr">
+        <is>
+          <t>-S, --search</t>
+        </is>
+      </c>
+      <c r="B44" s="21" t="inlineStr">
+        <is>
+          <t>引数に一致するテンプレ/ImageStream/コンテナイメージを検索</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="20" t="inlineStr">
+        <is>
+          <t>-L, --list</t>
+        </is>
+      </c>
+      <c r="B45" s="21" t="inlineStr">
+        <is>
+          <t>利用可能なローカルテンプレ・ImageStreamを一覧</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="20" t="inlineStr">
+        <is>
+          <t>--dry-run</t>
+        </is>
+      </c>
+      <c r="B46" s="21" t="inlineStr">
+        <is>
+          <t>実行せず結果のみ表示</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>-o, --output</t>
+        </is>
+      </c>
+      <c r="B47" s="21" t="inlineStr">
+        <is>
+          <t>出力形式（json/yaml/name/go-template/jsonpath 等）</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>--as-deployment-config</t>
+        </is>
+      </c>
+      <c r="B48" s="21" t="inlineStr">
+        <is>
+          <t>DeploymentConfig として作成（hooks/カスタム戦略が可能）</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="20" t="inlineStr">
+        <is>
+          <t>--as-test</t>
+        </is>
+      </c>
+      <c r="B49" s="21" t="inlineStr">
+        <is>
+          <t>テストデプロイとして作成（成功検証後スケールダウン）</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="20" t="inlineStr">
+        <is>
+          <t>--allow-missing-images</t>
+        </is>
+      </c>
+      <c r="B50" s="21" t="inlineStr">
+        <is>
+          <t>ローカル/レジストリで見つからない参照イメージも使用する</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="20" t="inlineStr">
+        <is>
+          <t>--allow-missing-imagestream-tags</t>
+        </is>
+      </c>
+      <c r="B51" s="21" t="inlineStr">
+        <is>
+          <t>存在しない ImageStream タグも使用する</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="20" t="inlineStr">
+        <is>
+          <t>--insecure-registry</t>
+        </is>
+      </c>
+      <c r="B52" s="21" t="inlineStr">
+        <is>
+          <t>参照イメージが安全でないレジストリ上として証明書検証をバイパス</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="20" t="inlineStr">
+        <is>
+          <t>--no-install</t>
+        </is>
+      </c>
+      <c r="B53" s="21" t="inlineStr">
+        <is>
+          <t>インストール可能と自称するイメージを実行しない</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="20" t="inlineStr">
+        <is>
+          <t>--grant-install-rights</t>
+        </is>
+      </c>
+      <c r="B54" s="21" t="inlineStr">
+        <is>
+          <t>アカウントへのアクセスが必要なコンポーネントにトークン使用を許可（信頼するイメージのみ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="20" t="inlineStr">
+        <is>
+          <t>--ignore-unknown-parameters</t>
+        </is>
+      </c>
+      <c r="B55" s="21" t="inlineStr">
+        <is>
+          <t>指定パラメータがテンプレートに無くても処理を継続</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="20" t="inlineStr">
+        <is>
+          <t>--allow-missing-template-keys</t>
+        </is>
+      </c>
+      <c r="B56" s="21" t="inlineStr">
+        <is>
+          <t>テンプレートのフィールド/キー欠落エラーを無視（golang/jsonpath出力のみ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="20" t="inlineStr">
+        <is>
+          <t>-a, --show-all / --show-labels / --show-managed-fields / --sort-by / --output-version</t>
+        </is>
+      </c>
+      <c r="B57" s="21" t="inlineStr">
+        <is>
+          <t>出力整形系オプション（全件表示/ラベル列/managedFields保持/ソート/APIバージョン指定）</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="18" t="inlineStr">
+        <is>
+          <t>oc get [TYPE[.VERSION][.GROUP]] [NAME | -l label] [flags]</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="28" customHeight="1">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>1つまたは複数のリソースを表示。ラベルセレクタで絞り込み可能。`oc api-resources` で対応リソース一覧。</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="19" t="inlineStr">
+        <is>
+          <t>オプション</t>
+        </is>
+      </c>
+      <c r="B61" s="19" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="20" t="inlineStr">
+        <is>
+          <t>-o, --output</t>
+        </is>
+      </c>
+      <c r="B62" s="21" t="inlineStr">
+        <is>
+          <t>出力形式（json/yaml/name/wide/custom-columns/jsonpath/go-template 等）</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="20" t="inlineStr">
+        <is>
+          <t>-w, --watch</t>
+        </is>
+      </c>
+      <c r="B63" s="21" t="inlineStr">
+        <is>
+          <t>取得後、変更を監視し続ける</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="20" t="inlineStr">
+        <is>
+          <t>--watch-only</t>
+        </is>
+      </c>
+      <c r="B64" s="21" t="inlineStr">
+        <is>
+          <t>一覧取得せず、変更のみ監視</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="20" t="inlineStr">
+        <is>
+          <t>--output-watch-events</t>
+        </is>
+      </c>
+      <c r="B65" s="21" t="inlineStr">
+        <is>
+          <t>--watch/--watch-only 時に watch イベントオブジェクトを出力</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="20" t="inlineStr">
+        <is>
+          <t>-l, --selector</t>
+        </is>
+      </c>
+      <c r="B66" s="21" t="inlineStr">
+        <is>
+          <t>ラベルセレクタで絞り込み（=, ==, !=, in, notin に対応）</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="20" t="inlineStr">
+        <is>
+          <t>--field-selector</t>
+        </is>
+      </c>
+      <c r="B67" s="21" t="inlineStr">
+        <is>
+          <t>フィールドセレクタで絞り込み（=, ==, != に対応）</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="20" t="inlineStr">
+        <is>
+          <t>-A, --all-namespaces</t>
+        </is>
+      </c>
+      <c r="B68" s="21" t="inlineStr">
+        <is>
+          <t>全namespaceを横断して一覧（現在contextのnamespaceは無視）</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="20" t="inlineStr">
+        <is>
+          <t>-f, --filename</t>
+        </is>
+      </c>
+      <c r="B69" s="21" t="inlineStr">
+        <is>
+          <t>対象リソースを識別するファイル/ディレクトリ/URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="20" t="inlineStr">
+        <is>
+          <t>-k, --kustomize</t>
+        </is>
+      </c>
+      <c r="B70" s="21" t="inlineStr">
+        <is>
+          <t>kustomization ディレクトリを処理（-f/-R と併用不可）</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="20" t="inlineStr">
+        <is>
+          <t>-R, --recursive</t>
+        </is>
+      </c>
+      <c r="B71" s="21" t="inlineStr">
+        <is>
+          <t>-f のディレクトリを再帰的に処理</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="20" t="inlineStr">
+        <is>
+          <t>-L, --label-columns</t>
+        </is>
+      </c>
+      <c r="B72" s="21" t="inlineStr">
+        <is>
+          <t>カンマ区切りのラベルを列として表示（大小区別あり）</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="20" t="inlineStr">
+        <is>
+          <t>--show-labels</t>
+        </is>
+      </c>
+      <c r="B73" s="21" t="inlineStr">
+        <is>
+          <t>全ラベルを最終列に表示</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="20" t="inlineStr">
+        <is>
+          <t>--show-kind</t>
+        </is>
+      </c>
+      <c r="B74" s="21" t="inlineStr">
+        <is>
+          <t>リソース種別を表示</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="20" t="inlineStr">
+        <is>
+          <t>--no-headers</t>
+        </is>
+      </c>
+      <c r="B75" s="21" t="inlineStr">
+        <is>
+          <t>default/custom-column出力時にヘッダーを表示しない</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="20" t="inlineStr">
+        <is>
+          <t>--sort-by</t>
+        </is>
+      </c>
+      <c r="B76" s="21" t="inlineStr">
+        <is>
+          <t>JSONPath式でソート（例 '{.metadata.name}'）</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="20" t="inlineStr">
+        <is>
+          <t>--ignore-not-found</t>
+        </is>
+      </c>
+      <c r="B77" s="21" t="inlineStr">
+        <is>
+          <t>対象が存在しない場合に NotFound エラーを抑制</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="20" t="inlineStr">
+        <is>
+          <t>--chunk-size</t>
+        </is>
+      </c>
+      <c r="B78" s="21" t="inlineStr">
+        <is>
+          <t>大きな一覧をチャンクで返す（既定500、0で無効。beta）</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="20" t="inlineStr">
+        <is>
+          <t>--subresource</t>
+        </is>
+      </c>
+      <c r="B79" s="21" t="inlineStr">
+        <is>
+          <t>指定リソースのサブリソースを取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="20" t="inlineStr">
+        <is>
+          <t>--raw</t>
+        </is>
+      </c>
+      <c r="B80" s="21" t="inlineStr">
+        <is>
+          <t>サーバーへリクエストする生のURI</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="20" t="inlineStr">
+        <is>
+          <t>--template</t>
+        </is>
+      </c>
+      <c r="B81" s="21" t="inlineStr">
+        <is>
+          <t>-o=go-template(-file) 時に使うテンプレート文字列/ファイルパス</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="20" t="inlineStr">
+        <is>
+          <t>--server-print</t>
+        </is>
+      </c>
+      <c r="B82" s="21" t="inlineStr">
+        <is>
+          <t>サーバー側でテーブル出力させる（拡張API/CRD対応。既定true）</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="20" t="inlineStr">
+        <is>
+          <t>--allow-missing-template-keys / --show-managed-fields</t>
+        </is>
+      </c>
+      <c r="B83" s="21" t="inlineStr">
+        <is>
+          <t>テンプレートキー欠落の無視（既定true）/ managedFields保持</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="18" t="inlineStr">
+        <is>
+          <t>oc create -f FILENAME [flags] / create &lt;subcommand&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="28" customHeight="1">
+      <c r="A86" s="17" t="inlineStr">
+        <is>
+          <t>ファイルやstdinからリソースを作成（JSON/YAML対応）。サブコマンドで個別リソースも作成可能。</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="19" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="B87" s="19" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="20" t="inlineStr">
+        <is>
+          <t>サブコマンド</t>
+        </is>
+      </c>
+      <c r="B88" s="21" t="inlineStr">
+        <is>
+          <t>build / clusterresourcequota / clusterrole / clusterrolebinding / configmap / cronjob / deployment / deploymentconfig / identity / imagestream / imagestreamtag / ingress / job / namespace / poddisruptionbudget / priorityclass / quota / role / rolebinding / route / secret / service / serviceaccount / token / user / useridentitymapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="20" t="inlineStr">
+        <is>
+          <t>-f, --filename</t>
+        </is>
+      </c>
+      <c r="B89" s="21" t="inlineStr">
+        <is>
+          <t>作成に使うファイル/ディレクトリ/URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="20" t="inlineStr">
+        <is>
+          <t>-k, --kustomize</t>
+        </is>
+      </c>
+      <c r="B90" s="21" t="inlineStr">
+        <is>
+          <t>kustomization ディレクトリを処理（-f/-R と併用不可）</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="20" t="inlineStr">
+        <is>
+          <t>-R, --recursive</t>
+        </is>
+      </c>
+      <c r="B91" s="21" t="inlineStr">
+        <is>
+          <t>-f のディレクトリを再帰的に処理</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="20" t="inlineStr">
+        <is>
+          <t>--edit</t>
+        </is>
+      </c>
+      <c r="B92" s="21" t="inlineStr">
+        <is>
+          <t>作成前に API リソースを編集</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="20" t="inlineStr">
+        <is>
+          <t>--dry-run</t>
+        </is>
+      </c>
+      <c r="B93" s="21" t="inlineStr">
+        <is>
+          <t>none|server|client。client=送信せず表示、server=永続化せずサーバー検証</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="20" t="inlineStr">
+        <is>
+          <t>--validate</t>
+        </is>
+      </c>
+      <c r="B94" s="21" t="inlineStr">
+        <is>
+          <t>strict(true)|warn|ignore(false)。スキーマ検証の挙動</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="20" t="inlineStr">
+        <is>
+          <t>--save-config</t>
+        </is>
+      </c>
+      <c r="B95" s="21" t="inlineStr">
+        <is>
+          <t>現在のオブジェクト構成をアノテーションに保存（将来の apply 用）</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="20" t="inlineStr">
+        <is>
+          <t>--field-manager</t>
+        </is>
+      </c>
+      <c r="B96" s="21" t="inlineStr">
+        <is>
+          <t>フィールド所有者追跡に使うマネージャ名（既定 'kubectl-create'）</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="20" t="inlineStr">
+        <is>
+          <t>-o, --output</t>
+        </is>
+      </c>
+      <c r="B97" s="21" t="inlineStr">
+        <is>
+          <t>出力形式（json/yaml/name/go-template/jsonpath 等）</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="20" t="inlineStr">
+        <is>
+          <t>-l, --selector</t>
+        </is>
+      </c>
+      <c r="B98" s="21" t="inlineStr">
+        <is>
+          <t>ラベルセレクタで絞り込み</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="20" t="inlineStr">
+        <is>
+          <t>--raw</t>
+        </is>
+      </c>
+      <c r="B99" s="21" t="inlineStr">
+        <is>
+          <t>サーバーへ POST する生のURI</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="20" t="inlineStr">
+        <is>
+          <t>--template / --allow-missing-template-keys / --show-managed-fields / --windows-line-endings</t>
+        </is>
+      </c>
+      <c r="B100" s="21" t="inlineStr">
+        <is>
+          <t>テンプレート/欠落キー無視/managedFields保持/改行コード（--edit時）</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="18" t="inlineStr">
+        <is>
+          <t>oc rollout SUBCOMMAND [flags]</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="28" customHeight="1">
+      <c r="A103" s="17" t="inlineStr">
+        <is>
+          <t>1つ以上のリソースのロールアウトを管理。対象: deployments / daemonsets / statefulsets / deploymentConfigs(非推奨)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="18" customHeight="1">
+      <c r="A104" s="19" t="inlineStr">
+        <is>
+          <t>サブコマンド</t>
+        </is>
+      </c>
+      <c r="B104" s="19" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="20" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B105" s="21" t="inlineStr">
+        <is>
+          <t>ロールアウトの状態を表示</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="20" t="inlineStr">
+        <is>
+          <t>history</t>
+        </is>
+      </c>
+      <c r="B106" s="21" t="inlineStr">
+        <is>
+          <t>ロールアウトの履歴を表示する</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="20" t="inlineStr">
+        <is>
+          <t>undo</t>
+        </is>
+      </c>
+      <c r="B107" s="21" t="inlineStr">
+        <is>
+          <t>現在のロールアウトを取り消す（前のデプロイへ戻す）</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="20" t="inlineStr">
+        <is>
+          <t>restart</t>
+        </is>
+      </c>
+      <c r="B108" s="21" t="inlineStr">
+        <is>
+          <t>リソースを再起動（--selector でラベル指定も可）</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="20" t="inlineStr">
+        <is>
+          <t>pause</t>
+        </is>
+      </c>
+      <c r="B109" s="21" t="inlineStr">
+        <is>
+          <t>対象リソースを一時停止としてマーク</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="20" t="inlineStr">
+        <is>
+          <t>resume</t>
+        </is>
+      </c>
+      <c r="B110" s="21" t="inlineStr">
+        <is>
+          <t>一時停止中のリソースを再開</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="20" t="inlineStr">
+        <is>
+          <t>cancel</t>
+        </is>
+      </c>
+      <c r="B111" s="21" t="inlineStr">
+        <is>
+          <t>進行中のデプロイをキャンセル</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="20" t="inlineStr">
+        <is>
+          <t>retry</t>
+        </is>
+      </c>
+      <c r="B112" s="21" t="inlineStr">
+        <is>
+          <t>直近の失敗したロールアウトを再試行</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="20" t="inlineStr">
+        <is>
+          <t>latest</t>
+        </is>
+      </c>
+      <c r="B113" s="21" t="inlineStr">
+        <is>
+          <t>トリガーの最新状態でDeploymentConfigの新規ロールアウトを開始</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="30" customHeight="1">
+      <c r="A115" s="9" t="inlineStr">
+        <is>
+          <t>※ 上記は提供された実機 `oc --help` 出力に忠実。各サブコマンドのさらに詳細なオプションは `oc &lt;command&gt; &lt;subcommand&gt; --help`、全コマンド共通のグローバルオプションは `oc options` を参照。</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="11" t="inlineStr">
+        <is>
+          <t>OpenShift Developer CLI コマンド: https://docs.openshift.com/container-platform/latest/cli_reference/openshift_cli/developer-cli-commands.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="11" t="inlineStr">
+        <is>
+          <t>kubectl コマンドリファレンス（共通オプション）: https://kubernetes.io/docs/reference/kubectl/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A86:B86"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="A85:B85"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A103:B103"/>
+    <mergeCell ref="A115:B115"/>
+    <mergeCell ref="A117:B117"/>
+    <mergeCell ref="A102:B102"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A118:B118"/>
+    <mergeCell ref="A22:B22"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(adhoc): expand command detail sheet with 8 more commands
実機oc --help出力に基づきstart-build/expose/scale/logs/rsh/exec/
debug/adm policyの全オプション詳細を⑥に追加。計13コマンドに拡充。

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai_generated/adhoc/openshift_kubernetes_comparison.xlsx
+++ b/ai_generated/adhoc/openshift_kubernetes_comparison.xlsx
@@ -3682,7 +3682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B118"/>
+  <dimension ref="A1:B252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3699,7 +3699,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>提供された実機の `oc &lt;command&gt; --help` 出力を忠実に転記。バージョン正確（実行環境の oc に準拠）。対象コマンド: login / new-app / get / create / rollout。（他コマンドの完全な詳細が必要な場合は、同様に oc &lt;command&gt; --help の出力を提供してください）</t>
+          <t>提供された実機の `oc &lt;command&gt; --help` 出力を忠実に転記。バージョン正確（実行環境の oc に準拠）。対象コマンド: login / new-app / get / create / rollout / start-build / expose / scale / logs / rsh / exec / debug / adm policy。（他コマンドの完全な詳細が必要な場合は、同様に oc &lt;command&gt; --help の出力を提供してください）</t>
         </is>
       </c>
     </row>
@@ -4925,44 +4925,1492 @@
         </is>
       </c>
     </row>
-    <row r="115" ht="30" customHeight="1">
-      <c r="A115" s="9" t="inlineStr">
+    <row r="115" ht="22" customHeight="1">
+      <c r="A115" s="18" t="inlineStr">
+        <is>
+          <t>oc start-build (BUILDCONFIG | --from-build=BUILD) [flags]</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="28" customHeight="1">
+      <c r="A116" s="17" t="inlineStr">
+        <is>
+          <t>指定ビルド設定で新規ビルドを開始、または --from-build=&lt;name&gt; で既存ビルドをコピー。--from-file/--from-dir/--from-repo でソースを直接渡せる。バイナリ入力のビルドはソースをサーバーに保持しない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="18" customHeight="1">
+      <c r="A117" s="19" t="inlineStr">
+        <is>
+          <t>オプション</t>
+        </is>
+      </c>
+      <c r="B117" s="19" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="20" t="inlineStr">
+        <is>
+          <t>--from-build</t>
+        </is>
+      </c>
+      <c r="B118" s="21" t="inlineStr">
+        <is>
+          <t>再実行するビルドの名前を指定</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="20" t="inlineStr">
+        <is>
+          <t>--from-dir</t>
+        </is>
+      </c>
+      <c r="B119" s="21" t="inlineStr">
+        <is>
+          <t>アーカイブしてバイナリ入力に使うディレクトリ</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="20" t="inlineStr">
+        <is>
+          <t>--from-file</t>
+        </is>
+      </c>
+      <c r="B120" s="21" t="inlineStr">
+        <is>
+          <t>バイナリ入力に使うファイル（pom.xml/Dockerfile等。ビルドソース中の唯一のファイルになる）</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="20" t="inlineStr">
+        <is>
+          <t>--from-repo</t>
+        </is>
+      </c>
+      <c r="B121" s="21" t="inlineStr">
+        <is>
+          <t>バイナリ入力に使うローカルソースリポジトリのパス</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="20" t="inlineStr">
+        <is>
+          <t>--from-archive</t>
+        </is>
+      </c>
+      <c r="B122" s="21" t="inlineStr">
+        <is>
+          <t>ビルド前に展開してバイナリ入力に使うアーカイブ（tar/tar.gz/zip）</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="20" t="inlineStr">
+        <is>
+          <t>--commit</t>
+        </is>
+      </c>
+      <c r="B123" s="21" t="inlineStr">
+        <is>
+          <t>ビルドが使うソースコミット識別子（Gitリポジトリベースのビルドが必要）</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="20" t="inlineStr">
+        <is>
+          <t>-F, --follow</t>
+        </is>
+      </c>
+      <c r="B124" s="21" t="inlineStr">
+        <is>
+          <t>ビルドを開始し、完了/失敗までログを追従</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="20" t="inlineStr">
+        <is>
+          <t>-w, --wait</t>
+        </is>
+      </c>
+      <c r="B125" s="21" t="inlineStr">
+        <is>
+          <t>ビルド完了を待機。失敗時は非ゼロ終了コードで終了</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="20" t="inlineStr">
+        <is>
+          <t>-e, --env</t>
+        </is>
+      </c>
+      <c r="B126" s="21" t="inlineStr">
+        <is>
+          <t>ビルドコンテナに設定する環境変数（KEY=VALUE）</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="20" t="inlineStr">
+        <is>
+          <t>--build-arg</t>
+        </is>
+      </c>
+      <c r="B127" s="21" t="inlineStr">
+        <is>
+          <t>ビルド時にDockerへ渡すKEY=VALUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="20" t="inlineStr">
+        <is>
+          <t>--build-loglevel</t>
+        </is>
+      </c>
+      <c r="B128" s="21" t="inlineStr">
+        <is>
+          <t>ビルドログ出力のログレベル</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="20" t="inlineStr">
+        <is>
+          <t>--exclude</t>
+        </is>
+      </c>
+      <c r="B129" s="21" t="inlineStr">
+        <is>
+          <t>--from-dir 時、ソースツリーから除外するファイルの正規表現（既定で .git を除外）</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="20" t="inlineStr">
+        <is>
+          <t>--incremental</t>
+        </is>
+      </c>
+      <c r="B130" s="21" t="inlineStr">
+        <is>
+          <t>source-strategyビルドの incremental 設定を上書き</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="20" t="inlineStr">
+        <is>
+          <t>--no-cache</t>
+        </is>
+      </c>
+      <c r="B131" s="21" t="inlineStr">
+        <is>
+          <t>docker-strategyビルドの noCache 設定を上書き</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="20" t="inlineStr">
+        <is>
+          <t>--from-webhook</t>
+        </is>
+      </c>
+      <c r="B132" s="21" t="inlineStr">
+        <is>
+          <t>既存ビルド設定をトリガーする汎用 webhook URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="20" t="inlineStr">
+        <is>
+          <t>--git-post-receive</t>
+        </is>
+      </c>
+      <c r="B133" s="21" t="inlineStr">
+        <is>
+          <t>ビルドをトリガーする post-receive フックの内容</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="20" t="inlineStr">
+        <is>
+          <t>--git-repository</t>
+        </is>
+      </c>
+      <c r="B134" s="21" t="inlineStr">
+        <is>
+          <t>post-receive 用 git リポジトリのパス（既定: カレント）</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="20" t="inlineStr">
+        <is>
+          <t>--list-webhooks</t>
+        </is>
+      </c>
+      <c r="B135" s="21" t="inlineStr">
+        <is>
+          <t>指定ビルド設定/ビルドの webhook 一覧（all / generic / github）</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="20" t="inlineStr">
+        <is>
+          <t>-o, --output / --template / --show-managed-fields / --allow-missing-template-keys</t>
+        </is>
+      </c>
+      <c r="B136" s="21" t="inlineStr">
+        <is>
+          <t>出力整形系</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="22" customHeight="1">
+      <c r="A138" s="18" t="inlineStr">
+        <is>
+          <t>oc expose (-f FILENAME | TYPE NAME) [flags]</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="28" customHeight="1">
+      <c r="A139" s="17" t="inlineStr">
+        <is>
+          <t>コンテナをServiceとして内部公開、またはRouteとして外部公開。dc/rc/service/pod を指定ポートで新規Serviceとして公開可能。ラベル未指定時は公開元のラベルを再利用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="18" customHeight="1">
+      <c r="A140" s="19" t="inlineStr">
+        <is>
+          <t>オプション</t>
+        </is>
+      </c>
+      <c r="B140" s="19" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="20" t="inlineStr">
+        <is>
+          <t>--name</t>
+        </is>
+      </c>
+      <c r="B141" s="21" t="inlineStr">
+        <is>
+          <t>新しく作成するオブジェクト名</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="20" t="inlineStr">
+        <is>
+          <t>--hostname</t>
+        </is>
+      </c>
+      <c r="B142" s="21" t="inlineStr">
+        <is>
+          <t>新規Routeのホスト名を設定</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="20" t="inlineStr">
+        <is>
+          <t>--path</t>
+        </is>
+      </c>
+      <c r="B143" s="21" t="inlineStr">
+        <is>
+          <t>新規Routeのパスを設定</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="20" t="inlineStr">
+        <is>
+          <t>--wildcard-policy</t>
+        </is>
+      </c>
+      <c r="B144" s="21" t="inlineStr">
+        <is>
+          <t>ホスト名のワイルドカードポリシー（None / Subdomain。既定 None）</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="20" t="inlineStr">
+        <is>
+          <t>--port</t>
+        </is>
+      </c>
+      <c r="B145" s="21" t="inlineStr">
+        <is>
+          <t>Serviceが提供するポート（未指定なら公開元からコピー）</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="20" t="inlineStr">
+        <is>
+          <t>--target-port</t>
+        </is>
+      </c>
+      <c r="B146" s="21" t="inlineStr">
+        <is>
+          <t>トラフィックを向けるコンテナ側ポート名/番号（任意）</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="20" t="inlineStr">
+        <is>
+          <t>--protocol</t>
+        </is>
+      </c>
+      <c r="B147" s="21" t="inlineStr">
+        <is>
+          <t>作成するServiceのネットワークプロトコル（既定 TCP）</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="20" t="inlineStr">
+        <is>
+          <t>--type</t>
+        </is>
+      </c>
+      <c r="B148" s="21" t="inlineStr">
+        <is>
+          <t>Service種別（ClusterIP / NodePort / LoadBalancer / ExternalName。既定 ClusterIP）</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="20" t="inlineStr">
+        <is>
+          <t>--cluster-ip</t>
+        </is>
+      </c>
+      <c r="B149" s="21" t="inlineStr">
+        <is>
+          <t>ServiceのClusterIP（空=自動割当、'None'=headless Service）</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="20" t="inlineStr">
+        <is>
+          <t>--external-ip</t>
+        </is>
+      </c>
+      <c r="B150" s="21" t="inlineStr">
+        <is>
+          <t>Serviceが受け付ける追加の外部IP（Kubernetes管理外）</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="20" t="inlineStr">
+        <is>
+          <t>--load-balancer-ip</t>
+        </is>
+      </c>
+      <c r="B151" s="21" t="inlineStr">
+        <is>
+          <t>LoadBalancerに割当てるIP（空ならエフェメラルIP）</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="20" t="inlineStr">
+        <is>
+          <t>--session-affinity</t>
+        </is>
+      </c>
+      <c r="B152" s="21" t="inlineStr">
+        <is>
+          <t>セッションアフィニティ（None / ClientIP）</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="20" t="inlineStr">
+        <is>
+          <t>--selector</t>
+        </is>
+      </c>
+      <c r="B153" s="21" t="inlineStr">
+        <is>
+          <t>Service用ラベルセレクタ（等価ベースのみ。空ならrc/replica setから推論）</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="20" t="inlineStr">
+        <is>
+          <t>-l, --labels</t>
+        </is>
+      </c>
+      <c r="B154" s="21" t="inlineStr">
+        <is>
+          <t>このコマンドで作成するServiceに付与するラベル</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="20" t="inlineStr">
+        <is>
+          <t>-f, --filename / -k, --kustomize / -R, --recursive</t>
+        </is>
+      </c>
+      <c r="B155" s="21" t="inlineStr">
+        <is>
+          <t>公開対象を識別する入力ファイル系</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="20" t="inlineStr">
+        <is>
+          <t>--dry-run / --save-config / --field-manager / --override-type / --overrides / -o / --template / --show-managed-fields</t>
+        </is>
+      </c>
+      <c r="B156" s="21" t="inlineStr">
+        <is>
+          <t>出力・上書き・整形系</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="22" customHeight="1">
+      <c r="A158" s="18" t="inlineStr">
+        <is>
+          <t>oc scale [--resource-version=v] [--current-replicas=n] --replicas=COUNT (-f FILENAME | TYPE NAME) [flags]</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="28" customHeight="1">
+      <c r="A159" s="17" t="inlineStr">
+        <is>
+          <t>deployment / replica set / replication controller / stateful set のサイズを変更。前提条件（--current-replicas / --resource-version）を満たす場合のみscale。</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="18" customHeight="1">
+      <c r="A160" s="19" t="inlineStr">
+        <is>
+          <t>オプション</t>
+        </is>
+      </c>
+      <c r="B160" s="19" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="20" t="inlineStr">
+        <is>
+          <t>--replicas</t>
+        </is>
+      </c>
+      <c r="B161" s="21" t="inlineStr">
+        <is>
+          <t>新しい希望レプリカ数（必須）</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="20" t="inlineStr">
+        <is>
+          <t>--current-replicas</t>
+        </is>
+      </c>
+      <c r="B162" s="21" t="inlineStr">
+        <is>
+          <t>現在サイズの前提条件。一致時のみscale（-1=条件なし）</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="20" t="inlineStr">
+        <is>
+          <t>--resource-version</t>
+        </is>
+      </c>
+      <c r="B163" s="21" t="inlineStr">
+        <is>
+          <t>resource version の前提条件。一致時のみscale</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="20" t="inlineStr">
+        <is>
+          <t>--all</t>
+        </is>
+      </c>
+      <c r="B164" s="21" t="inlineStr">
+        <is>
+          <t>指定リソース種別の、namespace内全リソースを選択</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="20" t="inlineStr">
+        <is>
+          <t>-f, --filename</t>
+        </is>
+      </c>
+      <c r="B165" s="21" t="inlineStr">
+        <is>
+          <t>サイズ変更対象を識別するファイル/ディレクトリ/URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="20" t="inlineStr">
+        <is>
+          <t>--timeout</t>
+        </is>
+      </c>
+      <c r="B166" s="21" t="inlineStr">
+        <is>
+          <t>scale操作を諦めるまでの待機時間（0=待たない。例 1s/2m/3h）</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="20" t="inlineStr">
+        <is>
+          <t>-l, --selector / -k, --kustomize / -R, --recursive</t>
+        </is>
+      </c>
+      <c r="B167" s="21" t="inlineStr">
+        <is>
+          <t>対象絞り込み・入力ファイル系</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="20" t="inlineStr">
+        <is>
+          <t>--dry-run / -o / --template / --show-managed-fields / --allow-missing-template-keys</t>
+        </is>
+      </c>
+      <c r="B168" s="21" t="inlineStr">
+        <is>
+          <t>出力・整形系</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="22" customHeight="1">
+      <c r="A170" s="18" t="inlineStr">
+        <is>
+          <t>oc logs [-f] [-p] (POD | TYPE/NAME) [-c CONTAINER] [flags]</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="28" customHeight="1">
+      <c r="A171" s="17" t="inlineStr">
+        <is>
+          <t>builds / build configs(bc) / deployment configs(dc) / pods のログを表示。複数コンテナ時は -c で指定、bc/dc は --version で版を指定。起動失敗時は --previous。</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="18" customHeight="1">
+      <c r="A172" s="19" t="inlineStr">
+        <is>
+          <t>オプション</t>
+        </is>
+      </c>
+      <c r="B172" s="19" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="20" t="inlineStr">
+        <is>
+          <t>-f, --follow</t>
+        </is>
+      </c>
+      <c r="B173" s="21" t="inlineStr">
+        <is>
+          <t>ログをストリーム（追従）する</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="20" t="inlineStr">
+        <is>
+          <t>-c, --container</t>
+        </is>
+      </c>
+      <c r="B174" s="21" t="inlineStr">
+        <is>
+          <t>このコンテナのログを表示</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="20" t="inlineStr">
+        <is>
+          <t>-p, --previous</t>
+        </is>
+      </c>
+      <c r="B175" s="21" t="inlineStr">
+        <is>
+          <t>Pod内コンテナの前回インスタンスのログ（存在すれば）</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="20" t="inlineStr">
+        <is>
+          <t>--all-containers</t>
+        </is>
+      </c>
+      <c r="B176" s="21" t="inlineStr">
+        <is>
+          <t>Pod内の全コンテナのログを取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="20" t="inlineStr">
+        <is>
+          <t>--all-pods</t>
+        </is>
+      </c>
+      <c r="B177" s="21" t="inlineStr">
+        <is>
+          <t>全Podからログ取得（prefix が true になる）</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="20" t="inlineStr">
+        <is>
+          <t>--tail</t>
+        </is>
+      </c>
+      <c r="B178" s="21" t="inlineStr">
+        <is>
+          <t>末尾N行を表示（既定-1。セレクタ無しで全行、セレクタ有りで10）</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="20" t="inlineStr">
+        <is>
+          <t>--since</t>
+        </is>
+      </c>
+      <c r="B179" s="21" t="inlineStr">
+        <is>
+          <t>相対時間より新しいログのみ（例 5s/2m/3h）。--since-time と排他</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="20" t="inlineStr">
+        <is>
+          <t>--since-time</t>
+        </is>
+      </c>
+      <c r="B180" s="21" t="inlineStr">
+        <is>
+          <t>指定日時(RFC3339)以降のログのみ。--since と排他</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="20" t="inlineStr">
+        <is>
+          <t>--timestamps</t>
+        </is>
+      </c>
+      <c r="B181" s="21" t="inlineStr">
+        <is>
+          <t>各行にタイムスタンプを付与</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="20" t="inlineStr">
+        <is>
+          <t>--limit-bytes</t>
+        </is>
+      </c>
+      <c r="B182" s="21" t="inlineStr">
+        <is>
+          <t>返すログの最大バイト数（既定: 無制限）</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="20" t="inlineStr">
+        <is>
+          <t>--prefix</t>
+        </is>
+      </c>
+      <c r="B183" s="21" t="inlineStr">
+        <is>
+          <t>各ログ行にログ元（pod名・コンテナ名）をプレフィックス</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="20" t="inlineStr">
+        <is>
+          <t>-l, --selector</t>
+        </is>
+      </c>
+      <c r="B184" s="21" t="inlineStr">
+        <is>
+          <t>ラベルセレクタで絞り込み</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="20" t="inlineStr">
+        <is>
+          <t>--max-log-requests</t>
+        </is>
+      </c>
+      <c r="B185" s="21" t="inlineStr">
+        <is>
+          <t>セレクタ使用時に追従する同時ログ数の最大（既定5）</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="20" t="inlineStr">
+        <is>
+          <t>--version</t>
+        </is>
+      </c>
+      <c r="B186" s="21" t="inlineStr">
+        <is>
+          <t>ビルド/デプロイの特定バージョンのログを表示（&gt;0）</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="20" t="inlineStr">
+        <is>
+          <t>--pod-running-timeout</t>
+        </is>
+      </c>
+      <c r="B187" s="21" t="inlineStr">
+        <is>
+          <t>少なくとも1Podが実行されるまで待つ時間（既定20s）</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="20" t="inlineStr">
+        <is>
+          <t>--ignore-errors</t>
+        </is>
+      </c>
+      <c r="B188" s="21" t="inlineStr">
+        <is>
+          <t>follow時に発生するエラーを非致命的として扱う</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="20" t="inlineStr">
+        <is>
+          <t>--insecure-skip-tls-verify-backend</t>
+        </is>
+      </c>
+      <c r="B189" s="21" t="inlineStr">
+        <is>
+          <t>ログ取得元 kubelet の身元検証をスキップ</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="22" customHeight="1">
+      <c r="A191" s="18" t="inlineStr">
+        <is>
+          <t>oc rsh [-c CONTAINER] [flags] (POD | TYPE/NAME) COMMAND [args...]</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="28" customHeight="1">
+      <c r="A192" s="17" t="inlineStr">
+        <is>
+          <t>コンテナへのリモートシェルセッションを開く。pods/dc/deployments/jobs/daemon sets/rc/replica sets に対応（pod以外はready podに解決）。既定シェルは /bin/sh。標準入力が対話的ならTTYを自動割当。シェルの無いコンテナは oc exec を使う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="18" customHeight="1">
+      <c r="A193" s="19" t="inlineStr">
+        <is>
+          <t>オプション</t>
+        </is>
+      </c>
+      <c r="B193" s="19" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="20" t="inlineStr">
+        <is>
+          <t>-c, --container</t>
+        </is>
+      </c>
+      <c r="B194" s="21" t="inlineStr">
+        <is>
+          <t>コンテナ名（既定: 最初のコンテナ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="20" t="inlineStr">
+        <is>
+          <t>-t, --tty</t>
+        </is>
+      </c>
+      <c r="B195" s="21" t="inlineStr">
+        <is>
+          <t>擬似端末(TTY)を強制割当</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="20" t="inlineStr">
+        <is>
+          <t>-T, --no-tty</t>
+        </is>
+      </c>
+      <c r="B196" s="21" t="inlineStr">
+        <is>
+          <t>擬似端末(TTY)割当を無効化</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="20" t="inlineStr">
+        <is>
+          <t>--shell</t>
+        </is>
+      </c>
+      <c r="B197" s="21" t="inlineStr">
+        <is>
+          <t>シェルコマンドのパス（既定 /bin/sh）</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="20" t="inlineStr">
+        <is>
+          <t>-f, --filename</t>
+        </is>
+      </c>
+      <c r="B198" s="21" t="inlineStr">
+        <is>
+          <t>rsh対象に使うファイル</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="20" t="inlineStr">
+        <is>
+          <t>--pod-running-timeout</t>
+        </is>
+      </c>
+      <c r="B199" s="21" t="inlineStr">
+        <is>
+          <t>少なくとも1Podが実行されるまで待つ時間（既定1m）</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" ht="22" customHeight="1">
+      <c r="A201" s="18" t="inlineStr">
+        <is>
+          <t>oc exec (POD | TYPE/NAME) [-c CONTAINER] [flags] -- COMMAND [args...]</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" ht="28" customHeight="1">
+      <c r="A202" s="17" t="inlineStr">
+        <is>
+          <t>コンテナ内でコマンドを実行する。コマンドにフラグが含まれる場合は -- で区切る。</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" ht="18" customHeight="1">
+      <c r="A203" s="19" t="inlineStr">
+        <is>
+          <t>オプション</t>
+        </is>
+      </c>
+      <c r="B203" s="19" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="20" t="inlineStr">
+        <is>
+          <t>-c, --container</t>
+        </is>
+      </c>
+      <c r="B204" s="21" t="inlineStr">
+        <is>
+          <t>コンテナ名（省略時は default-container アノテーション、または最初のコンテナ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="20" t="inlineStr">
+        <is>
+          <t>-i, --stdin</t>
+        </is>
+      </c>
+      <c r="B205" s="21" t="inlineStr">
+        <is>
+          <t>標準入力をコンテナに渡す</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="20" t="inlineStr">
+        <is>
+          <t>-t, --tty</t>
+        </is>
+      </c>
+      <c r="B206" s="21" t="inlineStr">
+        <is>
+          <t>標準入力をTTYにする</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="20" t="inlineStr">
+        <is>
+          <t>-q, --quiet</t>
+        </is>
+      </c>
+      <c r="B207" s="21" t="inlineStr">
+        <is>
+          <t>リモートセッションの出力のみ表示</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="20" t="inlineStr">
+        <is>
+          <t>-f, --filename</t>
+        </is>
+      </c>
+      <c r="B208" s="21" t="inlineStr">
+        <is>
+          <t>exec対象に使うファイル</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="20" t="inlineStr">
+        <is>
+          <t>--pod-running-timeout</t>
+        </is>
+      </c>
+      <c r="B209" s="21" t="inlineStr">
+        <is>
+          <t>少なくとも1Podが実行されるまで待つ時間（既定1m）</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" ht="22" customHeight="1">
+      <c r="A211" s="18" t="inlineStr">
+        <is>
+          <t>oc debug RESOURCE/NAME [ENV1=VAL1 ...] [-c CONTAINER] [flags] [-- COMMAND]</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" ht="28" customHeight="1">
+      <c r="A212" s="17" t="inlineStr">
+        <is>
+          <t>実行中アプリのデバッグ用シェルを起動。実行中Podのカーボンコピー（ラベル除去・command=/bin/sh・readiness/liveness無効）を作成。--as-user/--as-rootで実行ユーザー変更。node/istag/--image も対象可。コマンド完了/中断でdebug Podは削除。</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" ht="18" customHeight="1">
+      <c r="A213" s="19" t="inlineStr">
+        <is>
+          <t>オプション</t>
+        </is>
+      </c>
+      <c r="B213" s="19" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="20" t="inlineStr">
+        <is>
+          <t>--as-root</t>
+        </is>
+      </c>
+      <c r="B214" s="21" t="inlineStr">
+        <is>
+          <t>true でコンテナを root ユーザーとして実行</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="20" t="inlineStr">
+        <is>
+          <t>--as-user</t>
+        </is>
+      </c>
+      <c r="B215" s="21" t="inlineStr">
+        <is>
+          <t>特定UIDでコンテナ実行を試みる（管理者が制限する場合あり）</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="20" t="inlineStr">
+        <is>
+          <t>-c, --container</t>
+        </is>
+      </c>
+      <c r="B216" s="21" t="inlineStr">
+        <is>
+          <t>コンテナ名（既定: 最初のコンテナ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="20" t="inlineStr">
+        <is>
+          <t>--image</t>
+        </is>
+      </c>
+      <c r="B217" s="21" t="inlineStr">
+        <is>
+          <t>対象コンテナが使うイメージを上書き</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="20" t="inlineStr">
+        <is>
+          <t>--image-stream</t>
+        </is>
+      </c>
+      <c r="B218" s="21" t="inlineStr">
+        <is>
+          <t>デバッグイメージを含む image stream（namespace/name:tag）</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="20" t="inlineStr">
+        <is>
+          <t>--node-name</t>
+        </is>
+      </c>
+      <c r="B219" s="21" t="inlineStr">
+        <is>
+          <t>実行する特定ノードを指定（既定: 任意の有効ノード）</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="20" t="inlineStr">
+        <is>
+          <t>--to-namespace</t>
+        </is>
+      </c>
+      <c r="B220" s="21" t="inlineStr">
+        <is>
+          <t>Podを作成するnamespaceを上書き（--namespace の代わり）</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="20" t="inlineStr">
+        <is>
+          <t>--one-container</t>
+        </is>
+      </c>
+      <c r="B221" s="21" t="inlineStr">
+        <is>
+          <t>選択コンテナのみ実行し、他は削除</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="20" t="inlineStr">
+        <is>
+          <t>--preserve-pod</t>
+        </is>
+      </c>
+      <c r="B222" s="21" t="inlineStr">
+        <is>
+          <t>debugコマンド終了後もPodを削除しない</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="20" t="inlineStr">
+        <is>
+          <t>--keep-annotations</t>
+        </is>
+      </c>
+      <c r="B223" s="21" t="inlineStr">
+        <is>
+          <t>元のPodアノテーションを保持</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="20" t="inlineStr">
+        <is>
+          <t>--keep-labels</t>
+        </is>
+      </c>
+      <c r="B224" s="21" t="inlineStr">
+        <is>
+          <t>元のPodラベルを保持</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="20" t="inlineStr">
+        <is>
+          <t>--keep-init-containers</t>
+        </is>
+      </c>
+      <c r="B225" s="21" t="inlineStr">
+        <is>
+          <t>Podのinitコンテナを実行（既定true）</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="20" t="inlineStr">
+        <is>
+          <t>--keep-liveness / --keep-readiness / --keep-startup</t>
+        </is>
+      </c>
+      <c r="B226" s="21" t="inlineStr">
+        <is>
+          <t>元の liveness / readiness / startup プローブを保持</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="20" t="inlineStr">
+        <is>
+          <t>-I, --no-stdin</t>
+        </is>
+      </c>
+      <c r="B227" s="21" t="inlineStr">
+        <is>
+          <t>STDIN受け渡しを回避（コマンド未指定時は既定true）</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="20" t="inlineStr">
+        <is>
+          <t>-t, --tty / -T, --no-tty</t>
+        </is>
+      </c>
+      <c r="B228" s="21" t="inlineStr">
+        <is>
+          <t>TTYの強制割当 / 割当無効化</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="20" t="inlineStr">
+        <is>
+          <t>--dry-run / -o / -f / -k / -R / -q / --show-labels / --show-managed-fields / --template / --allow-missing-template-keys</t>
+        </is>
+      </c>
+      <c r="B229" s="21" t="inlineStr">
+        <is>
+          <t>出力・入力・整形系</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="22" customHeight="1">
+      <c r="A231" s="18" t="inlineStr">
+        <is>
+          <t>oc adm policy &lt;subcommand&gt; [flags]</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="28" customHeight="1">
+      <c r="A232" s="17" t="inlineStr">
+        <is>
+          <t>クラスタ上のポリシー（ユーザーに適用するロール/ポリシー）を割当・管理する。詳細は clusterroles / clusterrolebindings / roles / rolebindings / scc を get/describe で確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" ht="18" customHeight="1">
+      <c r="A233" s="19" t="inlineStr">
+        <is>
+          <t>サブコマンド</t>
+        </is>
+      </c>
+      <c r="B233" s="19" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="20" t="inlineStr">
+        <is>
+          <t>add-cluster-role-to-group</t>
+        </is>
+      </c>
+      <c r="B234" s="21" t="inlineStr">
+        <is>
+          <t>クラスタ全プロジェクトでグループにロールを追加</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="20" t="inlineStr">
+        <is>
+          <t>add-cluster-role-to-user</t>
+        </is>
+      </c>
+      <c r="B235" s="21" t="inlineStr">
+        <is>
+          <t>クラスタ全プロジェクトでユーザーにロールを追加</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="20" t="inlineStr">
+        <is>
+          <t>add-role-to-group</t>
+        </is>
+      </c>
+      <c r="B236" s="21" t="inlineStr">
+        <is>
+          <t>現プロジェクトでグループにロールを追加</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="20" t="inlineStr">
+        <is>
+          <t>add-role-to-user</t>
+        </is>
+      </c>
+      <c r="B237" s="21" t="inlineStr">
+        <is>
+          <t>現プロジェクトでユーザー/ServiceAccountにロールを追加</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="20" t="inlineStr">
+        <is>
+          <t>add-scc-to-group</t>
+        </is>
+      </c>
+      <c r="B238" s="21" t="inlineStr">
+        <is>
+          <t>グループに SecurityContextConstraints を追加</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="20" t="inlineStr">
+        <is>
+          <t>add-scc-to-user</t>
+        </is>
+      </c>
+      <c r="B239" s="21" t="inlineStr">
+        <is>
+          <t>ユーザー/ServiceAccount に SecurityContextConstraints を追加</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="20" t="inlineStr">
+        <is>
+          <t>remove-cluster-role-from-group</t>
+        </is>
+      </c>
+      <c r="B240" s="21" t="inlineStr">
+        <is>
+          <t>クラスタ全プロジェクトでグループからロールを削除</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="20" t="inlineStr">
+        <is>
+          <t>remove-cluster-role-from-user</t>
+        </is>
+      </c>
+      <c r="B241" s="21" t="inlineStr">
+        <is>
+          <t>クラスタ全プロジェクトでユーザーからロールを削除</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="20" t="inlineStr">
+        <is>
+          <t>remove-group / remove-user</t>
+        </is>
+      </c>
+      <c r="B242" s="21" t="inlineStr">
+        <is>
+          <t>プロジェクトからグループ / ユーザーを削除</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="20" t="inlineStr">
+        <is>
+          <t>remove-role-from-group / remove-role-from-user</t>
+        </is>
+      </c>
+      <c r="B243" s="21" t="inlineStr">
+        <is>
+          <t>プロジェクトでグループ / ユーザーからロールを削除</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="20" t="inlineStr">
+        <is>
+          <t>remove-scc-from-group / remove-scc-from-user</t>
+        </is>
+      </c>
+      <c r="B244" s="21" t="inlineStr">
+        <is>
+          <t>SCC からグループ / ユーザーを削除</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="20" t="inlineStr">
+        <is>
+          <t>scc-review</t>
+        </is>
+      </c>
+      <c r="B245" s="21" t="inlineStr">
+        <is>
+          <t>どの ServiceAccount が Pod を作成できるかを確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="20" t="inlineStr">
+        <is>
+          <t>scc-subject-review</t>
+        </is>
+      </c>
+      <c r="B246" s="21" t="inlineStr">
+        <is>
+          <t>ユーザーまたは ServiceAccount が Pod を作成できるかを確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="20" t="inlineStr">
+        <is>
+          <t>who-can</t>
+        </is>
+      </c>
+      <c r="B247" s="21" t="inlineStr">
+        <is>
+          <t>リソースに対し指定アクションを誰が実行できるか一覧表示</t>
+        </is>
+      </c>
+    </row>
+    <row r="249" ht="30" customHeight="1">
+      <c r="A249" s="9" t="inlineStr">
         <is>
           <t>※ 上記は提供された実機 `oc --help` 出力に忠実。各サブコマンドのさらに詳細なオプションは `oc &lt;command&gt; &lt;subcommand&gt; --help`、全コマンド共通のグローバルオプションは `oc options` を参照。</t>
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="11" t="inlineStr">
+    <row r="251">
+      <c r="A251" s="11" t="inlineStr">
         <is>
           <t>OpenShift Developer CLI コマンド: https://docs.openshift.com/container-platform/latest/cli_reference/openshift_cli/developer-cli-commands.html</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="11" t="inlineStr">
+    <row r="252">
+      <c r="A252" s="11" t="inlineStr">
         <is>
           <t>kubectl コマンドリファレンス（共通オプション）: https://kubernetes.io/docs/reference/kubectl/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="A4:B4"/>
+  <mergeCells count="31">
+    <mergeCell ref="A232:B232"/>
+    <mergeCell ref="A201:B201"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="A191:B191"/>
+    <mergeCell ref="A103:B103"/>
+    <mergeCell ref="A138:B138"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A252:B252"/>
+    <mergeCell ref="A212:B212"/>
+    <mergeCell ref="A158:B158"/>
+    <mergeCell ref="A192:B192"/>
+    <mergeCell ref="A139:B139"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A86:B86"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="A251:B251"/>
     <mergeCell ref="A85:B85"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A103:B103"/>
+    <mergeCell ref="A249:B249"/>
+    <mergeCell ref="A116:B116"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A159:B159"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A231:B231"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A171:B171"/>
+    <mergeCell ref="A170:B170"/>
     <mergeCell ref="A115:B115"/>
-    <mergeCell ref="A117:B117"/>
+    <mergeCell ref="A202:B202"/>
     <mergeCell ref="A102:B102"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A118:B118"/>
-    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A211:B211"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>